<commit_message>
Reconstruct LTR phylogenies >600 members
</commit_message>
<xml_diff>
--- a/tabular/reference/ervr/ervr_data.xlsx
+++ b/tabular/reference/ervr/ervr_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/ervr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF530490-6141-A046-B9CA-357EA67E0604}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE10E827-498B-2D49-989C-D61C90811426}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2220" yWindow="860" windowWidth="23060" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1240" yWindow="520" windowWidth="23060" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="included" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="137">
   <si>
     <t>sequenceID</t>
   </si>
@@ -251,9 +251,6 @@
     <t>ERV-3.Lambda.52</t>
   </si>
   <si>
-    <t>ERV-3.Lambda.57</t>
-  </si>
-  <si>
     <t>ERV-3.Lambda.40</t>
   </si>
   <si>
@@ -263,21 +260,9 @@
     <t>ERV-3.Lambda.74</t>
   </si>
   <si>
-    <t>ERV-1.Rho.Rb.31</t>
-  </si>
-  <si>
-    <t>ERV-1.Rho.Rb.39</t>
-  </si>
-  <si>
     <t>ERV-1.Zeta.HF.52A</t>
   </si>
   <si>
-    <t>ERV-1.Zeta.19</t>
-  </si>
-  <si>
-    <t>ERV-1.Zeta.35</t>
-  </si>
-  <si>
     <t>medium reiteration frequency repeat 101</t>
   </si>
   <si>
@@ -359,9 +344,6 @@
     <t>lineage_id</t>
   </si>
   <si>
-    <t>Unclassified</t>
-  </si>
-  <si>
     <t>ERV-1.Zeta.W9P.P</t>
   </si>
   <si>
@@ -371,33 +353,9 @@
     <t>HF</t>
   </si>
   <si>
-    <t>ERVR-1.Zeta.MER41</t>
-  </si>
-  <si>
-    <t>ERVR-1.Zeta.MER57</t>
-  </si>
-  <si>
-    <t>Rhoretrovirus</t>
-  </si>
-  <si>
     <t>ERVR-1.Theta.LOR1</t>
   </si>
   <si>
-    <t>ERVR-1.Theta.37</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.43</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.38</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER31</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER21</t>
-  </si>
-  <si>
     <t>ERVR-1.Zeta.MER83A</t>
   </si>
   <si>
@@ -419,36 +377,12 @@
     <t>excluded</t>
   </si>
   <si>
-    <t>ERVR-1.Theta.101</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER61</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER89</t>
-  </si>
-  <si>
-    <t>ERVR-1.Theta.MER34b</t>
-  </si>
-  <si>
-    <t>ERVR-1.Unclassified.MER4</t>
-  </si>
-  <si>
-    <t>ERVR-1.Unclassified.MER4b</t>
-  </si>
-  <si>
-    <t>ERVR-1.Unclassified.MER65</t>
-  </si>
-  <si>
     <t>ERVR-3.Lambda.70</t>
   </si>
   <si>
     <t>ERVR-3.Lambda.76</t>
   </si>
   <si>
-    <t>ERVR-3.Lambda.16A3</t>
-  </si>
-  <si>
     <t>ERV-1.Eta.E.HQ</t>
   </si>
   <si>
@@ -465,6 +399,48 @@
   </si>
   <si>
     <t>NK</t>
+  </si>
+  <si>
+    <t>sublineage</t>
+  </si>
+  <si>
+    <t>human endogenous retrovirus L68</t>
+  </si>
+  <si>
+    <t>HERV-L68</t>
+  </si>
+  <si>
+    <t>ERV-3.Sigma.57</t>
+  </si>
+  <si>
+    <t>Sigmaretrovirus</t>
+  </si>
+  <si>
+    <t>endogenous retrovirus L47</t>
+  </si>
+  <si>
+    <t>ERV-L47</t>
+  </si>
+  <si>
+    <t>ERV-3.Sigma</t>
+  </si>
+  <si>
+    <t>ERV-3.Sigma.47</t>
+  </si>
+  <si>
+    <t>ERVR-1.Theta.24.101</t>
+  </si>
+  <si>
+    <t>ERVR-1.Zeta.43</t>
+  </si>
+  <si>
+    <t>ERVR-1.Theta.24.MER89</t>
+  </si>
+  <si>
+    <t>ERV-3.Lambda.16A3</t>
+  </si>
+  <si>
+    <t>ERV-1.Zeta.HF.19</t>
   </si>
 </sst>
 </file>
@@ -630,7 +606,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="44">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -843,6 +819,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF8AD8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5FC79"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59996337778862885"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39994506668294322"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF85FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1007,7 +1013,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
@@ -1032,6 +1038,11 @@
     <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="43" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1077,7 +1088,37 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1092,7 +1133,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF85FF"/>
       <color rgb="FFFF8AD8"/>
+      <color rgb="FFD5FC79"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1403,7 +1446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB9083D8-DE01-F14E-ACB5-AF33867092C5}">
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:S38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.33203125" customWidth="1"/>
@@ -1424,7 +1467,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>45</v>
@@ -1433,13 +1476,13 @@
         <v>46</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>1</v>
@@ -1475,42 +1518,42 @@
         <v>69</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>140</v>
+        <v>56</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>117</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>62</v>
+        <v>56</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H2" s="2">
-        <v>6996</v>
+        <v>6896</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="13" t="s">
-        <v>35</v>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>111</v>
+        <v>8</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>2</v>
@@ -1533,38 +1576,36 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>138</v>
+        <v>26</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>132</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>125</v>
+        <v>26</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>125</v>
+        <v>77</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>143</v>
+        <v>98</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H3" s="2">
-        <v>6070</v>
+        <v>6639</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J3" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="9">
-        <v>16</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="1"/>
       <c r="L3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1586,34 +1627,34 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>74</v>
+        <v>34</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>134</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>143</v>
+        <v>98</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H4" s="2">
-        <v>5530</v>
+        <v>7048</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="2" t="s">
@@ -1637,34 +1678,34 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>78</v>
+        <v>23</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>107</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>58</v>
+        <v>23</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>142</v>
+        <v>97</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H5" s="2">
-        <v>9084</v>
+        <v>8120</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>115</v>
+        <v>21</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="2" t="s">
@@ -1690,23 +1731,23 @@
       <c r="A6" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>79</v>
+      <c r="B6" s="17" t="s">
+        <v>76</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>40</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H6" s="2">
         <v>4981</v>
@@ -1718,7 +1759,7 @@
         <v>35</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>2</v>
@@ -1739,30 +1780,30 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>80</v>
+        <v>25</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>133</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H7" s="2">
-        <v>5586</v>
+        <v>4798</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>6</v>
@@ -1770,7 +1811,9 @@
       <c r="J7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="K7" s="1"/>
+      <c r="K7" s="1" t="s">
+        <v>106</v>
+      </c>
       <c r="L7" s="2" t="s">
         <v>2</v>
       </c>
@@ -1792,28 +1835,28 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>81</v>
+        <v>38</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>118</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>61</v>
+        <v>38</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>104</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H8" s="2">
-        <v>6918</v>
+        <v>6996</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>6</v>
@@ -1821,7 +1864,9 @@
       <c r="J8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="K8" s="1"/>
+      <c r="K8" s="1" t="s">
+        <v>105</v>
+      </c>
       <c r="L8" s="2" t="s">
         <v>2</v>
       </c>
@@ -1841,40 +1886,38 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>71</v>
+        <v>36</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>136</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H9" s="2">
-        <v>4996</v>
+        <v>5586</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="K9" s="10">
-        <v>16</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K9" s="1"/>
       <c r="L9" s="2" t="s">
         <v>2</v>
       </c>
@@ -1896,34 +1939,34 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>72</v>
+        <v>42</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>108</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>142</v>
+        <v>98</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H10" s="2">
-        <v>3556</v>
+        <v>4285</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J10" s="13" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="2" t="s">
@@ -1947,34 +1990,34 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>73</v>
+        <v>43</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>109</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>142</v>
+        <v>98</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H11" s="2">
-        <v>5343</v>
+        <v>4880</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J11" s="13" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="2" t="s">
@@ -1998,34 +2041,34 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>75</v>
+        <v>44</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>110</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>142</v>
+        <v>98</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H12" s="2">
-        <v>3329</v>
+        <v>2880</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J12" s="13" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="2" t="s">
@@ -2038,7 +2081,7 @@
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
       <c r="Q12" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R12">
         <v>1</v>
@@ -2049,36 +2092,38 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>76</v>
+        <v>111</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>135</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>16</v>
+        <v>111</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>68</v>
+        <v>111</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>70</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H13" s="2">
-        <v>5685</v>
+        <v>6070</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J13" s="13" t="s">
+      <c r="J13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K13" s="1"/>
+      <c r="K13" s="9">
+        <v>16</v>
+      </c>
       <c r="L13" s="2" t="s">
         <v>2</v>
       </c>
@@ -2092,7 +2137,7 @@
         <v>5</v>
       </c>
       <c r="R13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S13" s="2" t="b">
         <v>1</v>
@@ -2100,36 +2145,38 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>118</v>
+        <v>11</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>71</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H14" s="2">
-        <v>4798</v>
+        <v>4996</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="K14" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="K14" s="10">
+        <v>16</v>
+      </c>
       <c r="L14" s="2" t="s">
         <v>2</v>
       </c>
@@ -2151,34 +2198,34 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>129</v>
+        <v>14</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>73</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H15" s="2">
-        <v>6639</v>
+        <v>5530</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>144</v>
+        <v>10</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="2" t="s">
@@ -2202,34 +2249,34 @@
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>130</v>
+        <v>12</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>72</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H16" s="2">
-        <v>5217</v>
+        <v>3556</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>144</v>
+        <v>10</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="2" t="s">
@@ -2253,34 +2300,34 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>131</v>
+        <v>15</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H17" s="2">
-        <v>7048</v>
+        <v>3329</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="J17" s="13" t="s">
-        <v>21</v>
+        <v>9</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" s="2" t="s">
@@ -2304,34 +2351,34 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>113</v>
+        <v>16</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>75</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>104</v>
+        <v>70</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H18" s="2">
-        <v>3944</v>
+        <v>5685</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" s="2" t="s">
@@ -2347,7 +2394,7 @@
         <v>5</v>
       </c>
       <c r="R18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S18" s="2" t="b">
         <v>1</v>
@@ -2355,34 +2402,34 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>114</v>
+        <v>17</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>104</v>
+        <v>70</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H19" s="2">
-        <v>7133</v>
+        <v>5023</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="K19" s="1"/>
       <c r="L19" s="2" t="s">
@@ -2406,34 +2453,34 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>122</v>
+        <v>18</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>116</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>104</v>
+        <v>70</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H20" s="2">
-        <v>4285</v>
+        <v>6189</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="2" t="s">
@@ -2457,34 +2504,34 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>123</v>
+        <v>13</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>126</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>104</v>
+        <v>65</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>126</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H21" s="2">
-        <v>4880</v>
+        <v>5343</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>35</v>
+        <v>127</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="2" t="s">
@@ -2508,36 +2555,32 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>124</v>
+        <v>129</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>131</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>44</v>
+        <v>129</v>
       </c>
       <c r="D22" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="H22" s="2">
-        <v>2880</v>
-      </c>
       <c r="I22" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K22" s="1"/>
+        <v>127</v>
+      </c>
       <c r="L22" s="2" t="s">
         <v>2</v>
       </c>
@@ -2548,7 +2591,7 @@
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
       <c r="Q22" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R22">
         <v>1</v>
@@ -2558,35 +2601,35 @@
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A23" s="8" t="s">
-        <v>17</v>
+      <c r="A23" s="14" t="s">
+        <v>32</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>136</v>
+        <v>32</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>114</v>
       </c>
       <c r="H23" s="2">
-        <v>5023</v>
+        <v>5217</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J23" s="13" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>122</v>
       </c>
       <c r="K23" s="1"/>
       <c r="L23" s="2" t="s">
@@ -2609,35 +2652,35 @@
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A24" s="8" t="s">
-        <v>18</v>
+      <c r="A24" s="14" t="s">
+        <v>19</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>137</v>
+        <v>19</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>101</v>
+      <c r="G24" s="12" t="s">
+        <v>114</v>
       </c>
       <c r="H24" s="2">
-        <v>6189</v>
+        <v>4936</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J24" s="13" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>122</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="2" t="s">
@@ -2660,39 +2703,37 @@
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A25" s="8" t="s">
-        <v>56</v>
+      <c r="A25" s="14" t="s">
+        <v>22</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>139</v>
+        <v>22</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>56</v>
+        <v>22</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>59</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>114</v>
       </c>
       <c r="H25" s="2">
-        <v>6896</v>
+        <v>1786</v>
       </c>
       <c r="I25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J25" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="J25" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K25" s="1"/>
       <c r="L25" s="2" t="s">
         <v>2</v>
       </c>
@@ -2706,42 +2747,42 @@
         <v>5</v>
       </c>
       <c r="R25">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="S25" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A26" s="8" t="s">
-        <v>23</v>
+      <c r="A26" s="14" t="s">
+        <v>24</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H26" s="2">
-        <v>8120</v>
+        <v>4060</v>
       </c>
       <c r="I26" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J26" s="13" t="s">
-        <v>21</v>
+      <c r="J26" s="2" t="s">
+        <v>122</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="2" t="s">
@@ -2764,35 +2805,35 @@
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A27" s="8" t="s">
-        <v>19</v>
+      <c r="A27" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>57</v>
+        <v>27</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>142</v>
+        <v>98</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H27" s="2">
-        <v>4936</v>
+        <v>933</v>
       </c>
       <c r="I27" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="2" t="s">
@@ -2815,35 +2856,35 @@
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A28" s="8" t="s">
-        <v>22</v>
+      <c r="A28" s="14" t="s">
+        <v>28</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>119</v>
+        <v>28</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>59</v>
+        <v>28</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>79</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H28" s="2">
-        <v>1786</v>
+        <v>4936</v>
       </c>
       <c r="I28" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="2" t="s">
@@ -2866,35 +2907,35 @@
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A29" s="8" t="s">
-        <v>24</v>
+      <c r="A29" s="14" t="s">
+        <v>29</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H29" s="2">
-        <v>4060</v>
+        <v>5356</v>
       </c>
       <c r="I29" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="2" t="s">
@@ -2917,35 +2958,35 @@
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A30" s="8" t="s">
-        <v>27</v>
+      <c r="A30" s="14" t="s">
+        <v>31</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>121</v>
+        <v>31</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H30" s="2">
-        <v>933</v>
+        <v>6758</v>
       </c>
       <c r="I30" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="K30" s="1"/>
       <c r="L30" s="2" t="s">
@@ -2968,35 +3009,35 @@
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A31" s="8" t="s">
-        <v>28</v>
+      <c r="A31" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>120</v>
+        <v>33</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>84</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H31" s="2">
-        <v>4936</v>
+        <v>4871</v>
       </c>
       <c r="I31" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="K31" s="1"/>
       <c r="L31" s="2" t="s">
@@ -3009,7 +3050,7 @@
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
       <c r="Q31" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R31">
         <v>1</v>
@@ -3019,35 +3060,35 @@
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A32" s="8" t="s">
-        <v>29</v>
+      <c r="A32" s="14" t="s">
+        <v>30</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>132</v>
+        <v>30</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H32" s="2">
-        <v>5356</v>
+        <v>6387</v>
       </c>
       <c r="I32" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="K32" s="1"/>
       <c r="L32" s="2" t="s">
@@ -3070,35 +3111,35 @@
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A33" s="8" t="s">
-        <v>30</v>
+      <c r="A33" s="14" t="s">
+        <v>31</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>133</v>
+        <v>31</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H33" s="2">
-        <v>6387</v>
+        <v>6758</v>
       </c>
       <c r="I33" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="2" t="s">
@@ -3121,35 +3162,35 @@
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
-        <v>31</v>
+      <c r="A34" s="14" t="s">
+        <v>37</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>134</v>
+        <v>37</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H34" s="2">
-        <v>6758</v>
+        <v>6918</v>
       </c>
       <c r="I34" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="2" t="s">
@@ -3172,35 +3213,35 @@
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A35" s="8" t="s">
-        <v>33</v>
+      <c r="A35" s="14" t="s">
+        <v>39</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>135</v>
+        <v>39</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="H35" s="2">
-        <v>4871</v>
+        <v>3944</v>
       </c>
       <c r="I35" s="6" t="s">
         <v>6</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="K35" s="1"/>
       <c r="L35" s="2" t="s">
@@ -3213,7 +3254,7 @@
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
       <c r="Q35" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R35">
         <v>1</v>
@@ -3222,16 +3263,164 @@
         <v>1</v>
       </c>
     </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A36" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H36" s="2">
+        <v>7133</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K36" s="1"/>
+      <c r="L36" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="R36">
+        <v>1</v>
+      </c>
+      <c r="S36" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A37" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G37" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H37" s="2">
+        <v>9084</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K37" s="1"/>
+      <c r="L37" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" s="2"/>
+      <c r="Q37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="R37">
+        <v>1</v>
+      </c>
+      <c r="S37" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A38" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K38" s="1"/>
+      <c r="L38" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2"/>
+      <c r="Q38" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="R38">
+        <v>1</v>
+      </c>
+      <c r="S38" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S35">
-    <sortCondition ref="G2:G35"/>
-    <sortCondition ref="F2:F35"/>
-    <sortCondition ref="I2:I35"/>
-    <sortCondition ref="J2:J35"/>
-    <sortCondition ref="K2:K35"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S38">
+    <sortCondition ref="G2:G38"/>
+    <sortCondition ref="I2:I38"/>
+    <sortCondition ref="J2:J38"/>
+    <sortCondition ref="K2:K38"/>
   </sortState>
-  <conditionalFormatting sqref="R36:R1048576">
-    <cfRule type="colorScale" priority="97">
+  <conditionalFormatting sqref="R39:R1048576">
+    <cfRule type="colorScale" priority="107">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3243,7 +3432,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R1">
-    <cfRule type="colorScale" priority="39">
+    <cfRule type="colorScale" priority="49">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3255,7 +3444,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1">
-    <cfRule type="colorScale" priority="21">
+    <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3266,13 +3455,64 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G35">
-    <cfRule type="containsText" dxfId="0" priority="15" operator="containsText" text="excluded">
+  <conditionalFormatting sqref="G23:G36 G2:G21">
+    <cfRule type="containsText" dxfId="3" priority="25" operator="containsText" text="excluded">
       <formula>NOT(ISERROR(SEARCH("excluded",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R35">
-    <cfRule type="colorScale" priority="103">
+  <conditionalFormatting sqref="Q25">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R26:R30 S38 R32:R36 R2:R24">
+    <cfRule type="colorScale" priority="128">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G22">
+    <cfRule type="containsText" dxfId="2" priority="6" operator="containsText" text="excluded">
+      <formula>NOT(ISERROR(SEARCH("excluded",G22)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R37">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G37">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="excluded">
+      <formula>NOT(ISERROR(SEARCH("excluded",G37)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G38">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="excluded">
+      <formula>NOT(ISERROR(SEARCH("excluded",G38)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R31">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
Add LTRs to multi-LTR ERVR references
</commit_message>
<xml_diff>
--- a/tabular/reference/ervr/ervr_data.xlsx
+++ b/tabular/reference/ervr/ervr_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/ervr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126249C9-5552-5D47-8374-1FE771EEA27B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFAA139-C061-3045-A2EE-DBEF080874F4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="500" windowWidth="27860" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4740" yWindow="1640" windowWidth="27860" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="included" sheetId="2" r:id="rId1"/>

</xml_diff>